<commit_message>
feat: add complete collections library workflow
</commit_message>
<xml_diff>
--- a/workbook testings/padhivu_starter_populated (1) (1) (1).xlsx
+++ b/workbook testings/padhivu_starter_populated (1) (1) (1).xlsx
@@ -620,7 +620,7 @@
         <v>updatedAt</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-07-19T10:20:29.029Z</v>
+        <v>2026-07-19T11:59:44.359Z</v>
       </c>
     </row>
   </sheetData>
@@ -1569,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1649,9 +1649,61 @@
         <v>self-help</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>b87c24a4-86fd-4adc-b8ae-cbfe0e660a3d</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Series</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Love Death + Robots</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Netflix</v>
+      </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Watching</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>Animated Anthology</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>70114ea3-5ae5-4492-8438-96779f475055</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Book</v>
+      </c>
+      <c r="C5" t="str">
+        <v>A Man called Ove</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Fredrick Backmann</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Finished</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Amazing book to read</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Book, Feel Good</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>